<commit_message>
:up: algumas palavras tentadas
</commit_message>
<xml_diff>
--- a/banco_de_dados/vocabulario.xlsx
+++ b/banco_de_dados/vocabulario.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D64"/>
+  <dimension ref="A1:D77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -495,7 +495,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5">
@@ -515,7 +515,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -535,7 +535,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">
@@ -555,7 +555,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -575,7 +575,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9">
@@ -615,7 +615,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -635,7 +635,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12">
@@ -655,7 +655,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13">
@@ -715,7 +715,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="16">
@@ -755,7 +755,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18">
@@ -795,7 +795,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="20">
@@ -835,7 +835,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -855,7 +855,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23">
@@ -875,7 +875,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="24">
@@ -935,7 +935,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27">
@@ -975,7 +975,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29">
@@ -995,7 +995,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="30">
@@ -1035,7 +1035,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="32">
@@ -1055,7 +1055,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33">
@@ -1095,7 +1095,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35">
@@ -1155,7 +1155,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="38">
@@ -1195,7 +1195,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="40">
@@ -1215,7 +1215,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="41">
@@ -1315,7 +1315,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="46">
@@ -1335,7 +1335,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47">
@@ -1355,7 +1355,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="48">
@@ -1415,7 +1415,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="51">
@@ -1695,6 +1695,266 @@
         </is>
       </c>
       <c r="D64" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Yield</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>noun</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>rendimento, produção</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Stuck</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>noun</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>preso</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>likely</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>adverb</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>provavelmente</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>household names</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>expression</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>nomes muitos conhecidos</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>entrepreneur</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>noun</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>empreendedor</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>whether</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>conjunction</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>se</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>catch on</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>verb</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>tornar-se popular</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>lick</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>verb</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>lamber</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>morph</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>verb</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>transformar-se</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>stick</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>verb</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>grudar</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>doggedly</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>adverb</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>com tenacidade</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>flawed</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>adjective</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>imperfeito</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>venture</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>noun</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>risco, empreendimento</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
:up: algumas tentativas de respostas
</commit_message>
<xml_diff>
--- a/banco_de_dados/vocabulario.xlsx
+++ b/banco_de_dados/vocabulario.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D77"/>
+  <dimension ref="A1:D72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -475,7 +475,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -495,7 +495,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
@@ -521,7 +521,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>gums</t>
+          <t>periodontitis</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -531,17 +531,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>gengivas</t>
+          <t>periodontite</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>periodontitis</t>
+          <t>tissues</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -551,17 +551,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>periodontite</t>
+          <t>tecidos</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>periodontium</t>
+          <t>absence</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -571,37 +571,37 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>periodonto</t>
+          <t>ausência</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>tissues</t>
+          <t>regardless</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>noun</t>
+          <t>adverb</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>tecidos</t>
+          <t>sem considerar</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>absence</t>
+          <t>injury</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -611,127 +611,127 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ausência</t>
+          <t>ferida</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>plaque</t>
+          <t>likewise</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>noun</t>
+          <t>adjective</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>placa</t>
+          <t>da mesma maneira</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>regardless</t>
+          <t>hence</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>adverb</t>
+          <t>conjunction</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>sem considerar</t>
+          <t>por isso</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>injury</t>
+          <t>enhance</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>noun</t>
+          <t>verb</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>ferida</t>
+          <t>melhorar</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>likewise</t>
+          <t>likelihood</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>adjective</t>
+          <t>noun</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>da mesma maneira</t>
+          <t>probabilidade</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>hence</t>
+          <t>led</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>conjunction</t>
+          <t>adjective</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>por isso</t>
+          <t>liderado</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>enhance</t>
+          <t>bowel</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>verb</t>
+          <t>noun</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>melhorar</t>
+          <t>intestino</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -741,7 +741,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>likelihood</t>
+          <t>kidney</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -751,57 +751,57 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>probabilidade</t>
+          <t>rim</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>led</t>
+          <t>long-standing</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>adjective</t>
+          <t>phrasal adjective</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>liderado</t>
+          <t>de longa data</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>furthermore</t>
+          <t>maelstrom</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>conjunction</t>
+          <t>noun</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>além disso</t>
+          <t>redemoinho</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>bowel</t>
+          <t>underpinning</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -811,87 +811,87 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>intestino</t>
+          <t>sustentação</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>kidney</t>
+          <t>broadly</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>noun</t>
+          <t>adverb</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>rim</t>
+          <t>amplamente</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>long-standing</t>
+          <t>to struggle</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>phrasal adjective</t>
+          <t>verb</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>de longa data</t>
+          <t>lutar</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>maelstrom</t>
+          <t>booming</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>noun</t>
+          <t>verb</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>redemoinho</t>
+          <t>crescendo</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>underpinning</t>
+          <t>tailoring</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>noun</t>
+          <t>verb</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>sustentação</t>
+          <t>adaptando, alfaiataria</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -901,47 +901,47 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>broadly</t>
+          <t>railways</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>adverb</t>
+          <t>noun</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>amplamente</t>
+          <t>ferrovias</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>to struggle</t>
+          <t>rail travel</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>verb</t>
+          <t>noun</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>lutar</t>
+          <t>viagens de trem</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>booming</t>
+          <t>to shape</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -951,37 +951,37 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>crescendo</t>
+          <t>moldar</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>tailoring</t>
+          <t>pivotal</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>verb</t>
+          <t>adjective</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>adaptando, alfaiataria</t>
+          <t>fundamental</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>railways</t>
+          <t>billing</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -991,17 +991,17 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>ferrovias</t>
+          <t>cobrança</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>rail travel</t>
+          <t>patches</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1011,37 +1011,37 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>viagens de trem</t>
+          <t>remendos</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>to shape</t>
+          <t>enhanced</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>verb</t>
+          <t>adjective</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>moldar</t>
+          <t>aprimorada</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>pivotal</t>
+          <t>embedded</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1051,7 +1051,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>fundamental</t>
+          <t>integrado</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -1061,27 +1061,27 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>billing</t>
+          <t>to infer</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>noun</t>
+          <t>verb</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>cobrança</t>
+          <t>inferir</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>patches</t>
+          <t>scarce</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1091,147 +1091,147 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>remendos</t>
+          <t>escasso</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>enhanced</t>
+          <t>despite</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>adjective</t>
+          <t>preposition</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>aprimorada</t>
+          <t>apesar de</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>embedded</t>
+          <t>to threaten</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>adjective</t>
+          <t>preposition</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>integrado</t>
+          <t>ameaçar</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>to infer</t>
+          <t>leverage</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>verb</t>
+          <t>preposition</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>inferir</t>
+          <t>alavancar, aproveitar</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>scarce</t>
+          <t>coerced</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>noun</t>
+          <t>verb</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>escasso</t>
+          <t>coagido</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>despite</t>
+          <t>deemed</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>preposition</t>
+          <t>verb</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>apesar de</t>
+          <t>considerado</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>to threaten</t>
+          <t>attire</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>preposition</t>
+          <t>noun</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>ameaçar</t>
+          <t>traje</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>leverage</t>
+          <t>scapegoating</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>preposition</t>
+          <t>noun</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>alavancar, aproveitar</t>
+          <t>bode expiatório</t>
         </is>
       </c>
       <c r="D41" t="n">
@@ -1241,47 +1241,47 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>coerced</t>
+          <t>ostracization</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>verb</t>
+          <t>noun</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>coagido</t>
+          <t>ostracismo</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>deemed</t>
+          <t>aftermath</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>verb</t>
+          <t>noun</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>considerado</t>
+          <t>consequências</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>attire</t>
+          <t>conflation</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1291,7 +1291,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>traje</t>
+          <t>confusão</t>
         </is>
       </c>
       <c r="D44" t="n">
@@ -1301,37 +1301,37 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>scapegoating</t>
+          <t>virulent</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>noun</t>
+          <t>adjective</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>bode expiatório</t>
+          <t>virulento</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>ostracization</t>
+          <t>strikingly</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>noun</t>
+          <t>adverb</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>ostracismo</t>
+          <t>surpreendentemente</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -1341,7 +1341,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>aftermath</t>
+          <t>fodder</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1351,27 +1351,27 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>consequências</t>
+          <t>alimento, forragem</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>conflation</t>
+          <t>sheer</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>noun</t>
+          <t>adjective</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>confusão</t>
+          <t>puro</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1381,17 +1381,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>virulent</t>
+          <t>emblem</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>adjective</t>
+          <t>noun</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>virulento</t>
+          <t>emblema</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1401,37 +1401,37 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>to pose</t>
+          <t>Negroes</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>verb</t>
+          <t>noun</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>representar, posar</t>
+          <t>Negros</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>strikingly</t>
+          <t>enslavement</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>adverb</t>
+          <t>noun</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>surpreendentemente</t>
+          <t>escravização</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -1441,7 +1441,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>fodder</t>
+          <t>brand</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1451,7 +1451,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>alimento, forragem</t>
+          <t>tipo, marca</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -1461,7 +1461,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>sheer</t>
+          <t>unshackled</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1471,7 +1471,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>puro</t>
+          <t>livre</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -1481,7 +1481,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>emblem</t>
+          <t>infringement</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1491,7 +1491,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>emblema</t>
+          <t>violação</t>
         </is>
       </c>
       <c r="D54" t="n">
@@ -1501,17 +1501,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Negroes</t>
+          <t>inextricable</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>noun</t>
+          <t>adjective</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Negros</t>
+          <t>inextricável</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -1521,7 +1521,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>enslavement</t>
+          <t>outrage</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>escravização</t>
+          <t>ultraje</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -1541,7 +1541,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>brand</t>
+          <t>vitriol</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1551,7 +1551,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>tipo, marca</t>
+          <t>vitríolo</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -1561,17 +1561,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>unshackled</t>
+          <t>towards</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>adjective</t>
+          <t>preposition</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>livre</t>
+          <t>em relação</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -1581,17 +1581,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>infringement</t>
+          <t>refrain</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>noun</t>
+          <t>verb</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>violação</t>
+          <t>abster</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -1601,17 +1601,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>inextricable</t>
+          <t>Yield</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>adjective</t>
+          <t>noun</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>inextricável</t>
+          <t>rendimento, produção</t>
         </is>
       </c>
       <c r="D60" t="n">
@@ -1621,7 +1621,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>outrage</t>
+          <t>Stuck</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1631,7 +1631,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>ultraje</t>
+          <t>preso</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -1641,17 +1641,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>vitriol</t>
+          <t>likely</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>noun</t>
+          <t>adverb</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>vitríolo</t>
+          <t>provavelmente</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -1661,17 +1661,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>towards</t>
+          <t>household names</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>preposition</t>
+          <t>expression</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>em relação</t>
+          <t>nomes muitos conhecidos</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -1681,17 +1681,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>refrain</t>
+          <t>entrepreneur</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>verb</t>
+          <t>noun</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>abster</t>
+          <t>empreendedor</t>
         </is>
       </c>
       <c r="D64" t="n">
@@ -1701,17 +1701,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Yield</t>
+          <t>whether</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>noun</t>
+          <t>conjunction</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>rendimento, produção</t>
+          <t>se</t>
         </is>
       </c>
       <c r="D65" t="n">
@@ -1721,17 +1721,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Stuck</t>
+          <t>catch on</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>noun</t>
+          <t>verb</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>preso</t>
+          <t>tornar-se popular</t>
         </is>
       </c>
       <c r="D66" t="n">
@@ -1741,17 +1741,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>likely</t>
+          <t>lick</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>adverb</t>
+          <t>verb</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>provavelmente</t>
+          <t>lamber</t>
         </is>
       </c>
       <c r="D67" t="n">
@@ -1761,17 +1761,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>household names</t>
+          <t>morph</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>expression</t>
+          <t>verb</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>nomes muitos conhecidos</t>
+          <t>transformar-se</t>
         </is>
       </c>
       <c r="D68" t="n">
@@ -1781,17 +1781,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>entrepreneur</t>
+          <t>stick</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>noun</t>
+          <t>verb</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>empreendedor</t>
+          <t>grudar</t>
         </is>
       </c>
       <c r="D69" t="n">
@@ -1801,17 +1801,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>whether</t>
+          <t>doggedly</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>conjunction</t>
+          <t>adverb</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>se</t>
+          <t>com tenacidade</t>
         </is>
       </c>
       <c r="D70" t="n">
@@ -1821,17 +1821,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>catch on</t>
+          <t>flawed</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>verb</t>
+          <t>adjective</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>tornar-se popular</t>
+          <t>imperfeito</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -1841,120 +1841,20 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>lick</t>
+          <t>venture</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>verb</t>
+          <t>noun</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>lamber</t>
+          <t>risco, empreendimento</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>morph</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>verb</t>
-        </is>
-      </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>transformar-se</t>
-        </is>
-      </c>
-      <c r="D73" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>stick</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>verb</t>
-        </is>
-      </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>grudar</t>
-        </is>
-      </c>
-      <c r="D74" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>doggedly</t>
-        </is>
-      </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>adverb</t>
-        </is>
-      </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>com tenacidade</t>
-        </is>
-      </c>
-      <c r="D75" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>flawed</t>
-        </is>
-      </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>adjective</t>
-        </is>
-      </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>imperfeito</t>
-        </is>
-      </c>
-      <c r="D76" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>venture</t>
-        </is>
-      </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>noun</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>risco, empreendimento</t>
-        </is>
-      </c>
-      <c r="D77" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>